<commit_message>
S162: neutral site names + pickups from the customer's own sites (DEC-210)
300 sites named <CITY> <KIND> (no company names — seed test enforces it);
each customer owns 4 ship-from sites in 4 cities, index-assigned, none
shared; every pickup comes from them, deliveries never do. faker's
arrayElement takes one draw for any list >= 2 (verified in 9.9.0), so
0 shipment/order ids moved. Tests, fixtures and the Cognizant progression
example values follow (sheets regenerated, audit clean). Reseed owed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/story-packs/orders-search-progression.xlsx
+++ b/docs/story-packs/orders-search-progression.xlsx
@@ -872,7 +872,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>G2O TECH SOLUTIONS, Bastrop, LA, US</t>
+          <t>BASTROP TERMINAL, Bastrop, LA, US</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>SOLVAY CHEMICALS PL, Green River, WY, US</t>
+          <t>GREEN RIVER TERMINAL, Green River, WY, US</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">

</xml_diff>